<commit_message>
feat: add pivot table to Excel template
</commit_message>
<xml_diff>
--- a/experiments/templates/experiments-report-template.xlsx
+++ b/experiments/templates/experiments-report-template.xlsx
@@ -1,31 +1,63 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\source\cd-app\transcription-evals\experiments\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C7B4141-7C60-4509-8949-5EF5F8B01CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB22B8A-8FF2-40A1-ACE1-9B9B03734D1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="63120" yWindow="5685" windowWidth="31785" windowHeight="22920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="31920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Outputs" sheetId="1" r:id="rId1"/>
+    <sheet name="WER" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
+  <pivotCaches>
+    <pivotCache cacheId="12" r:id="rId3"/>
+  </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+  <si>
+    <t>reference_file</t>
+  </si>
+  <si>
+    <t>model_name</t>
+  </si>
+  <si>
+    <t>model_label</t>
+  </si>
+  <si>
+    <t>wer</t>
+  </si>
+  <si>
+    <t>mer</t>
+  </si>
+  <si>
+    <t>wil</t>
+  </si>
+  <si>
+    <t>cer</t>
+  </si>
+  <si>
+    <t>normalized_wer</t>
+  </si>
+  <si>
+    <t>normalized_mer</t>
+  </si>
+  <si>
+    <t>normalized_wil</t>
+  </si>
+  <si>
+    <t>normalized_cer</t>
+  </si>
   <si>
     <t>audio_file_name</t>
   </si>
@@ -33,37 +65,19 @@
     <t>audio_file_duration</t>
   </si>
   <si>
-    <t>model_name</t>
-  </si>
-  <si>
-    <t>model_label</t>
-  </si>
-  <si>
-    <t>wer</t>
-  </si>
-  <si>
-    <t>mer</t>
-  </si>
-  <si>
-    <t>wil</t>
-  </si>
-  <si>
-    <t>cer</t>
-  </si>
-  <si>
-    <t>normalized_wer</t>
-  </si>
-  <si>
-    <t>normalized_mer</t>
-  </si>
-  <si>
-    <t>normalized_wil</t>
-  </si>
-  <si>
-    <t>normalized_cer</t>
-  </si>
-  <si>
-    <t>reference_file</t>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>StdDev(WER)</t>
+  </si>
+  <si>
+    <t>Avg(WER)</t>
+  </si>
+  <si>
+    <t>Avg(normalized WER)</t>
+  </si>
+  <si>
+    <t>StdDev of normalized_wer</t>
   </si>
 </sst>
 </file>
@@ -113,16 +127,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -133,6 +159,197 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Yves P. Tkaczyk" refreshedDate="46070.716968171299" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{B7A2FA60-0A92-4B22-ADDF-8406A2E64B15}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:M99" sheet="Outputs"/>
+  </cacheSource>
+  <cacheFields count="13">
+    <cacheField name="reference_file" numFmtId="0">
+      <sharedItems containsNonDate="0" containsBlank="1" count="6">
+        <m/>
+        <s v="sample-01.json" u="1"/>
+        <s v="sample-02.json" u="1"/>
+        <s v="sample-03.json" u="1"/>
+        <s v="sample-04.json" u="1"/>
+        <s v="sample-05.json" u="1"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="model_name" numFmtId="0">
+      <sharedItems containsNonDate="0" containsBlank="1" count="3">
+        <m/>
+        <s v="AssemblyAI" u="1"/>
+        <s v="Deepgram" u="1"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="model_label" numFmtId="0">
+      <sharedItems containsNonDate="0" containsBlank="1" count="2">
+        <m/>
+        <s v="v3" u="1"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="wer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="mer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="wil" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="cer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="normalized_wer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="normalized_mer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="normalized_wil" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="normalized_cer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="audio_file_name" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="audio_file_duration" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="1">
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{39524549-1B91-461F-8C2F-46922AA341E6}" name="PivotTable1" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showError="1" showMissing="0" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A5:E5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="13">
+    <pivotField axis="axisRow" showAll="0" measureFilter="1">
+      <items count="7">
+        <item m="1" x="1"/>
+        <item m="1" x="2"/>
+        <item m="1" x="3"/>
+        <item m="1" x="4"/>
+        <item m="1" x="5"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item m="1" x="1"/>
+        <item m="1" x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item m="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="3">
+    <field x="1"/>
+    <field x="2"/>
+    <field x="0"/>
+  </rowFields>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+  </colItems>
+  <dataFields count="4">
+    <dataField name="Avg(WER)" fld="3" subtotal="average" baseField="0" baseItem="0" numFmtId="10"/>
+    <dataField name="StdDev(WER)" fld="3" subtotal="stdDev" baseField="0" baseItem="0"/>
+    <dataField name="Avg(normalized WER)" fld="7" subtotal="average" baseField="0" baseItem="0" numFmtId="10"/>
+    <dataField name="StdDev of normalized_wer" fld="7" subtotal="stdDev" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="0" type="valueGreaterThanOrEqual" evalOrder="-1" id="1" iMeasureFld="0">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <customFilters>
+            <customFilter operator="greaterThanOrEqual" val="0"/>
+          </customFilters>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -404,49 +621,98 @@
     <col min="1" max="14" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7CAF51C-88F5-4682-841E-A7C0517B9B4E}">
+  <dimension ref="A5:E5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="11" width="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>